<commit_message>
JDBC:implementada toda la ampliación con checklist
</commit_message>
<xml_diff>
--- a/checklist.xlsx
+++ b/checklist.xlsx
@@ -1709,7 +1709,11 @@
       <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="21"/>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E4" s="22"/>
     </row>
     <row r="5" spans="1:5">
@@ -1722,7 +1726,11 @@
       <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="28"/>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E5" s="22"/>
     </row>
     <row r="6" spans="1:5">
@@ -1735,7 +1743,11 @@
       <c r="C6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="28"/>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" ht="27.6">
@@ -1748,7 +1760,11 @@
       <c r="C7" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D7" s="10"/>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="27"/>
@@ -1767,7 +1783,11 @@
       <c r="C10" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="11"/>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
@@ -1779,7 +1799,11 @@
       <c r="C11" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="15"/>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
@@ -1791,7 +1815,11 @@
       <c r="C12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="15"/>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="9" t="s">
@@ -1803,7 +1831,11 @@
       <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="12"/>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="D14" s="4"/>
@@ -1823,7 +1855,11 @@
       <c r="C16" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="33"/>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:4" ht="41.4">
       <c r="A17" s="7" t="s">
@@ -1835,7 +1871,11 @@
       <c r="C17" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D17" s="32"/>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18" spans="1:4" ht="27.6">
       <c r="A18" s="7" t="s">
@@ -1847,7 +1887,11 @@
       <c r="C18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="15"/>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="7" t="s">
@@ -1859,7 +1903,11 @@
       <c r="C19" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="15"/>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
@@ -1871,7 +1919,11 @@
       <c r="C20" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="12"/>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2"/>
@@ -1889,7 +1941,11 @@
       <c r="C23" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D23" s="11"/>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="7" t="s">
@@ -1901,7 +1957,11 @@
       <c r="C24" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D24" s="15"/>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:4" ht="27.6">
       <c r="A25" s="9" t="s">
@@ -1913,7 +1973,11 @@
       <c r="C25" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D25" s="15"/>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
@@ -1925,7 +1989,11 @@
       <c r="C26" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="D26" s="12"/>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28" spans="1:4">
       <c r="C28" s="6" t="s">
@@ -1942,7 +2010,11 @@
       <c r="C29" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="18"/>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="7" t="s">
@@ -1954,7 +2026,11 @@
       <c r="C30" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="15"/>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
@@ -1966,7 +2042,11 @@
       <c r="C31" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="D31" s="12"/>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:4">
       <c r="C33" s="6" t="s">
@@ -1983,7 +2063,11 @@
       <c r="C34" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="D34" s="26"/>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="36" spans="1:4">
       <c r="C36" s="6" t="s">
@@ -2000,7 +2084,11 @@
       <c r="C37" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D37" s="18"/>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="9" t="s">
@@ -2012,7 +2100,11 @@
       <c r="C38" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="D38" s="25"/>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="40" spans="1:4">
       <c r="C40" s="6" t="s">
@@ -2029,7 +2121,11 @@
       <c r="C41" t="s">
         <v>67</v>
       </c>
-      <c r="D41" s="11"/>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="9" t="s">
@@ -2041,7 +2137,11 @@
       <c r="C42" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="D42" s="15"/>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="9" t="s">
@@ -2053,7 +2153,11 @@
       <c r="C43" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D43" s="15"/>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="9" t="s">
@@ -2065,7 +2169,11 @@
       <c r="C44" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="D44" s="25"/>
+      <c r="D44" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="46" spans="1:4">
       <c r="C46" s="6" t="s">
@@ -2082,7 +2190,11 @@
       <c r="C47" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D47" s="11"/>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="48" spans="1:4" ht="27.6">
       <c r="A48" s="7" t="s">
@@ -2094,7 +2206,11 @@
       <c r="C48" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D48" s="15"/>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="9" t="s">
@@ -2106,7 +2222,11 @@
       <c r="C49" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D49" s="15"/>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="7" t="s">
@@ -2118,7 +2238,11 @@
       <c r="C50" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D50" s="15"/>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="9" t="s">
@@ -2130,7 +2254,11 @@
       <c r="C51" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D51" s="15"/>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="9" t="s">
@@ -2142,7 +2270,11 @@
       <c r="C52" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D52" s="12"/>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="54" spans="1:4">
       <c r="C54" s="6" t="s">
@@ -2159,7 +2291,11 @@
       <c r="C55" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D55" s="11"/>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="9" t="s">
@@ -2171,7 +2307,11 @@
       <c r="C56" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D56" s="12"/>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="57" spans="1:4">
       <c r="C57" s="4"/>
@@ -2192,7 +2332,11 @@
       <c r="C59" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D59" s="26"/>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="60" spans="1:4">
       <c r="C60" s="4"/>
@@ -2214,7 +2358,11 @@
       <c r="C62" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D62" s="11"/>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="7" t="s">
@@ -2226,7 +2374,11 @@
       <c r="C63" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D63" s="15"/>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="9" t="s">
@@ -2238,7 +2390,11 @@
       <c r="C64" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D64" s="15"/>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="7" t="s">
@@ -2250,7 +2406,11 @@
       <c r="C65" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D65" s="15"/>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E65" s="4"/>
     </row>
     <row r="66" spans="1:5">
@@ -2263,7 +2423,11 @@
       <c r="C66" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D66" s="15"/>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="67" spans="1:5" ht="27.6">
       <c r="A67" s="9" t="s">
@@ -2275,7 +2439,11 @@
       <c r="C67" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D67" s="12"/>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="68" spans="1:5">
       <c r="C68" s="4"/>
@@ -2302,7 +2470,11 @@
       <c r="C71" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D71" s="26"/>
+      <c r="D71" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="2"/>
@@ -2344,7 +2516,11 @@
       <c r="C4" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="D4" s="21"/>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E4" s="22"/>
     </row>
     <row r="5" spans="1:5">
@@ -2357,7 +2533,11 @@
       <c r="C5" s="36" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="28"/>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E5" s="22"/>
     </row>
     <row r="6" spans="1:5">
@@ -2370,7 +2550,11 @@
       <c r="C6" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="28"/>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" ht="27.6">
@@ -2383,7 +2567,11 @@
       <c r="C7" s="38" t="s">
         <v>144</v>
       </c>
-      <c r="D7" s="10"/>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="27"/>
@@ -2402,7 +2590,11 @@
       <c r="C10" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="11"/>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
@@ -2414,7 +2606,11 @@
       <c r="C11" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="15"/>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
@@ -2426,7 +2622,11 @@
       <c r="C12" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="D12" s="15"/>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="9" t="s">
@@ -2438,7 +2638,11 @@
       <c r="C13" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="D13" s="12"/>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="C14" s="35"/>
@@ -2459,7 +2663,11 @@
       <c r="C16" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="D16" s="33"/>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:4" ht="41.4">
       <c r="A17" s="7" t="s">
@@ -2471,7 +2679,11 @@
       <c r="C17" s="36" t="s">
         <v>147</v>
       </c>
-      <c r="D17" s="32"/>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18" spans="1:4" ht="27.6">
       <c r="A18" s="7" t="s">
@@ -2483,7 +2695,11 @@
       <c r="C18" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="D18" s="15"/>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="7" t="s">
@@ -2495,7 +2711,11 @@
       <c r="C19" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="D19" s="15"/>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
@@ -2507,7 +2727,11 @@
       <c r="C20" s="44" t="s">
         <v>106</v>
       </c>
-      <c r="D20" s="12"/>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2"/>
@@ -2525,7 +2749,11 @@
       <c r="C23" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="D23" s="11"/>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="7" t="s">
@@ -2537,7 +2765,11 @@
       <c r="C24" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="15"/>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:4" ht="27.6">
       <c r="A25" s="9" t="s">
@@ -2549,7 +2781,11 @@
       <c r="C25" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="D25" s="15"/>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
@@ -2561,7 +2797,11 @@
       <c r="C26" s="44" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="12"/>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28" spans="1:4">
       <c r="C28" s="40" t="s">
@@ -2578,7 +2818,11 @@
       <c r="C29" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="D29" s="18"/>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="7" t="s">
@@ -2590,7 +2834,11 @@
       <c r="C30" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="15"/>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
@@ -2602,7 +2850,11 @@
       <c r="C31" s="44" t="s">
         <v>149</v>
       </c>
-      <c r="D31" s="12"/>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:4">
       <c r="C33" s="40" t="s">
@@ -2619,7 +2871,11 @@
       <c r="C34" s="45" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="26"/>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="36" spans="1:4">
       <c r="C36" s="40" t="s">
@@ -2636,7 +2892,11 @@
       <c r="C37" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="D37" s="18"/>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="9" t="s">
@@ -2648,7 +2908,11 @@
       <c r="C38" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="D38" s="25"/>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="40" spans="1:4">
       <c r="C40" s="40" t="s">
@@ -2665,7 +2929,11 @@
       <c r="C41" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="D41" s="11"/>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="9" t="s">
@@ -2677,7 +2945,11 @@
       <c r="C42" s="46" t="s">
         <v>121</v>
       </c>
-      <c r="D42" s="15"/>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="43" spans="1:4" ht="27.6">
       <c r="A43" s="9" t="s">
@@ -2689,7 +2961,11 @@
       <c r="C43" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="D43" s="15"/>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="9" t="s">
@@ -2701,7 +2977,11 @@
       <c r="C44" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="D44" s="25"/>
+      <c r="D44" s="25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="46" spans="1:4">
       <c r="C46" s="40" t="s">
@@ -2718,7 +2998,11 @@
       <c r="C47" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="D47" s="11"/>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="48" spans="1:4" ht="27.6">
       <c r="A48" s="7" t="s">
@@ -2730,7 +3014,11 @@
       <c r="C48" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="D48" s="15"/>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="9" t="s">
@@ -2742,7 +3030,11 @@
       <c r="C49" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="D49" s="15"/>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="7" t="s">
@@ -2754,7 +3046,11 @@
       <c r="C50" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="D50" s="15"/>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="9" t="s">
@@ -2766,7 +3062,11 @@
       <c r="C51" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="D51" s="15"/>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="9" t="s">
@@ -2778,7 +3078,11 @@
       <c r="C52" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="D52" s="12"/>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="54" spans="1:4">
       <c r="C54" s="40" t="s">
@@ -2795,7 +3099,11 @@
       <c r="C55" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="D55" s="11"/>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="9" t="s">
@@ -2807,7 +3115,11 @@
       <c r="C56" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="D56" s="12"/>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="57" spans="1:4">
       <c r="C57" s="39"/>
@@ -2828,7 +3140,11 @@
       <c r="C59" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="D59" s="26"/>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="60" spans="1:4">
       <c r="C60" s="39"/>
@@ -2850,7 +3166,11 @@
       <c r="C62" s="39" t="s">
         <v>134</v>
       </c>
-      <c r="D62" s="11"/>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="7" t="s">
@@ -2862,7 +3182,11 @@
       <c r="C63" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="D63" s="15"/>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="9" t="s">
@@ -2874,7 +3198,11 @@
       <c r="C64" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="D64" s="15"/>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="7" t="s">
@@ -2886,7 +3214,11 @@
       <c r="C65" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="D65" s="15"/>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="E65" s="4"/>
     </row>
     <row r="66" spans="1:5">
@@ -2899,7 +3231,11 @@
       <c r="C66" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="D66" s="15"/>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="67" spans="1:5" ht="27.6">
       <c r="A67" s="9" t="s">
@@ -2911,7 +3247,11 @@
       <c r="C67" s="38" t="s">
         <v>139</v>
       </c>
-      <c r="D67" s="12"/>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="68" spans="1:5">
       <c r="C68" s="39"/>
@@ -2939,7 +3279,11 @@
       <c r="C71" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="D71" s="26"/>
+      <c r="D71" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="2"/>

</xml_diff>